<commit_message>
Chemistry: ubot (unbottled) water → tap, never bottled
ubot = UN-bottled, so it cannot be مياه شرب/معبأة. classify() now converts any
ubot sample that resolved to bottled/drinking (generic/blank/wash-water names,
some via earlier corrections) to مياه الحنفية (tap). Filter and non-potable
subtypes untouched. ubot bottled 25→0; tap 555→580.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/clean/chemistry/chem_water_analysis_2024.xlsx
+++ b/clean/chemistry/chem_water_analysis_2024.xlsx
@@ -1711,7 +1711,7 @@
       </c>
       <c r="BD8" t="inlineStr">
         <is>
-          <t>مياه شرب/معبأة</t>
+          <t>مياه الحنفية</t>
         </is>
       </c>
       <c r="BF8" t="inlineStr">
@@ -2760,7 +2760,7 @@
       </c>
       <c r="BD16" t="inlineStr">
         <is>
-          <t>مياه شرب/معبأة</t>
+          <t>مياه الحنفية</t>
         </is>
       </c>
       <c r="BF16" t="inlineStr">
@@ -3808,7 +3808,7 @@
       </c>
       <c r="BD24" t="inlineStr">
         <is>
-          <t>مياه شرب/معبأة</t>
+          <t>مياه الحنفية</t>
         </is>
       </c>
       <c r="BF24" t="inlineStr">
@@ -4201,7 +4201,7 @@
       </c>
       <c r="BD27" t="inlineStr">
         <is>
-          <t>مياه شرب/معبأة</t>
+          <t>مياه الحنفية</t>
         </is>
       </c>
       <c r="BF27" t="inlineStr">
@@ -4332,7 +4332,7 @@
       </c>
       <c r="BD28" t="inlineStr">
         <is>
-          <t>مياه شرب/معبأة</t>
+          <t>مياه الحنفية</t>
         </is>
       </c>
       <c r="BF28" t="inlineStr">

</xml_diff>